<commit_message>
scalebay update 2026-09-14 01:55 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-15 02:32 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-15 15:01 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-16 03:27 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-16 15:55 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-17 04:18 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-18 05:11 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-18 17:41 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-19 06:11 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-19 18:42 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-20 07:06 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-21 08:02 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-21 20:30 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-22 08:40 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-22 23:06 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-23 11:39 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-24 00:08 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-25 01:03 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-26 02:03 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-26 14:37 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-27 03:17 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-27 15:46 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-30 05:33 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-30 18:03 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-01 06:33 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-02 07:16 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-02 19:51 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-03 08:19 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-03 20:52 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-04 21:45 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-05 10:13 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-05 22:49 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-07 00:00 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-08 01:07 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-08 13:37 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-09 15:27 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-10 03:55 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-11 17:59 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-12 06:10 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-13 06:52 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-14 09:10 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-14 21:48 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-15 09:55 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-18 00:27 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-19 15:33 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-20 03:39 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-21 04:57 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-22 05:55 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-22 18:21 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-23 06:51 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-23 19:20 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-25 21:28 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-27 10:48 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-27 23:20 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-30 01:30 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-10-31 02:24 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>